<commit_message>
Bottle servo push test
</commit_message>
<xml_diff>
--- a/SLSS V5/SLSS V5 Requirements.xlsx
+++ b/SLSS V5/SLSS V5 Requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\Documents\SLSS\SLSS V5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A29BB5A-0008-4A04-A30B-AA14578E7230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75C21136-2A8E-4D75-B304-3A610453EB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="48">
   <si>
     <t>No</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>two spaced beams which can wrap string around to hang the substrate from</t>
+  </si>
+  <si>
+    <t>Check hole size of adafruit temperature and humidity sensor</t>
   </si>
 </sst>
 </file>
@@ -212,21 +215,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill>
@@ -284,13 +273,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E8483FE8-83BD-4FD4-B975-1BFA0938C5BF}" name="Table1" displayName="Table1" ref="B14:E32" totalsRowShown="0" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E8483FE8-83BD-4FD4-B975-1BFA0938C5BF}" name="Table1" displayName="Table1" ref="B14:E32" totalsRowShown="0" dataDxfId="8">
   <autoFilter ref="B14:E32" xr:uid="{E8483FE8-83BD-4FD4-B975-1BFA0938C5BF}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{23CFA789-FF03-475E-AA4D-506F8D054482}" name="No." dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{D749B61C-74C6-4654-8692-591DC432ABF2}" name="Requirement" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{5BA96E61-7E13-4B39-B5AB-BBD799D8FADB}" name="Solution/design consideration" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{91BF3BD5-542B-4D71-AB6F-75648DBB12C6}" name="Agreed Consideration" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{23CFA789-FF03-475E-AA4D-506F8D054482}" name="No." dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D749B61C-74C6-4654-8692-591DC432ABF2}" name="Requirement" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{5BA96E61-7E13-4B39-B5AB-BBD799D8FADB}" name="Solution/design consideration" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{91BF3BD5-542B-4D71-AB6F-75648DBB12C6}" name="Agreed Consideration" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -852,10 +841,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15:E32">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",E15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",E15)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -940,7 +929,12 @@
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="2:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C7" s="1"/>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="D7" s="1"/>
     </row>
   </sheetData>
@@ -957,10 +951,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E7">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="No">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",E3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Yes">
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Yes">
       <formula>NOT(ISERROR(SEARCH("Yes",E3)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>